<commit_message>
restore lost work due to git hub messed up
</commit_message>
<xml_diff>
--- a/LvM_Refed_TAGkinetics_portalAAs_SCFAs/LvM_refed_TAGkinetics_hpAAs_SCFAs.xlsx
+++ b/LvM_Refed_TAGkinetics_portalAAs_SCFAs/LvM_refed_TAGkinetics_hpAAs_SCFAs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/boyuan/Desktop/Harvard/Research/Energy Metabolism Atlas/LvM_Refed_TAGkinetics_portalAAs_SCFAs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EA9DC8F-778E-6440-9464-8044625F2A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE6CB8C-FD4A-B14D-A01D-843996B089B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17400" activeTab="1" xr2:uid="{5E0D7404-E754-4442-97F6-BA3E5E250F0E}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{5E0D7404-E754-4442-97F6-BA3E5E250F0E}"/>
   </bookViews>
   <sheets>
     <sheet name="LvM" sheetId="37" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="213">
   <si>
     <t>enzyme</t>
   </si>
@@ -1733,7 +1733,113 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>E</t>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>C</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>D</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>H</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>I</t>
+    </r>
+  </si>
+  <si>
+    <t>TAGLino.Lv -&gt; AcCoA.Lv</t>
+  </si>
+  <si>
+    <t>TAGLino is treatd as a "substrate", and Lino.Blood-&gt;TAGLino should not be included in the network</t>
+  </si>
+  <si>
+    <r>
+      <t>13C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>LinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>H</t>
     </r>
     <r>
       <rPr>
@@ -1763,7 +1869,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>F</t>
+      <t>O</t>
     </r>
     <r>
       <rPr>
@@ -1793,7 +1899,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>G</t>
+      <t>P</t>
     </r>
     <r>
       <rPr>
@@ -1823,7 +1929,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>H</t>
+      <t>Q</t>
     </r>
     <r>
       <rPr>
@@ -1853,7 +1959,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>I</t>
+      <t>R</t>
     </r>
     <r>
       <rPr>
@@ -1883,7 +1989,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>J</t>
+      <t>S</t>
     </r>
     <r>
       <rPr>
@@ -1896,6 +2002,36 @@
   </si>
   <si>
     <r>
+      <t>13C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>LinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>T</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>13CLinoKin</t>
     </r>
     <r>
@@ -1905,7 +2041,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>B</t>
+      <t>O</t>
     </r>
   </si>
   <si>
@@ -1919,7 +2055,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>C</t>
+      <t>P</t>
     </r>
   </si>
   <si>
@@ -1933,7 +2069,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>D</t>
+      <t>Q</t>
     </r>
   </si>
   <si>
@@ -1947,7 +2083,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>E</t>
+      <t>R</t>
     </r>
   </si>
   <si>
@@ -1961,7 +2097,7 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>F</t>
+      <t>S</t>
     </r>
   </si>
   <si>
@@ -1975,56 +2111,8 @@
         <color rgb="FF00B0F0"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>G</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>H</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>I</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>J</t>
-    </r>
-  </si>
-  <si>
-    <t>TAGLino.Lv -&gt; AcCoA.Lv</t>
-  </si>
-  <si>
-    <t>TAGLino is treatd as a "substrate", and Lino.Blood-&gt;TAGLino should not be included in the network</t>
+      <t>T</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3086,14 +3174,14 @@
         <v>11</v>
       </c>
       <c r="B12" s="56" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C12" s="57" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="62"/>
       <c r="E12" s="58" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -4400,7 +4488,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6AE8287-079C-D041-8E27-642CD2612D07}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="3.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
@@ -4455,7 +4543,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <f t="shared" ref="A4:A30" si="0">A3</f>
+        <f t="shared" ref="A4:A32" si="0">A3</f>
         <v>101</v>
       </c>
       <c r="B4" s="11" t="s">
@@ -4735,7 +4823,7 @@
         <v>16</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -4750,7 +4838,7 @@
         <v>16</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -4765,7 +4853,7 @@
         <v>16</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -4774,13 +4862,13 @@
         <v>101</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -4789,13 +4877,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -4804,13 +4892,13 @@
         <v>101</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -4819,13 +4907,13 @@
         <v>101</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -4834,13 +4922,13 @@
         <v>101</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -4849,13 +4937,43 @@
         <v>101</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <f t="shared" si="0"/>
+        <v>101</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <f t="shared" si="0"/>
+        <v>101</v>
+      </c>
+      <c r="B32" s="7" t="s">
         <v>206</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correct mouse id for refed-SCFA-hpAA-TAGkinetics full model; simplify refed LvM basic model network by removing fatty acids related reactions
</commit_message>
<xml_diff>
--- a/LvM_Refed_TAGkinetics_portalAAs_SCFAs/LvM_refed_TAGkinetics_hpAAs_SCFAs.xlsx
+++ b/LvM_Refed_TAGkinetics_portalAAs_SCFAs/LvM_refed_TAGkinetics_hpAAs_SCFAs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/boyuan/Desktop/Harvard/Research/Energy Metabolism Atlas/LvM_Refed_TAGkinetics_portalAAs_SCFAs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hui Lab\Desktop\liver_MFA\LvM_Refed_TAGkinetics_portalAAs_SCFAs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE6CB8C-FD4A-B14D-A01D-843996B089B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E88927B9-BDA1-4B0B-BE7F-1EE1FCD16D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{5E0D7404-E754-4442-97F6-BA3E5E250F0E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{5E0D7404-E754-4442-97F6-BA3E5E250F0E}"/>
   </bookViews>
   <sheets>
     <sheet name="LvM" sheetId="37" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="209">
   <si>
     <t>enzyme</t>
   </si>
@@ -1581,6 +1581,55 @@
     </r>
   </si>
   <si>
+    <t>TAGLino.Lv -&gt; AcCoA.Lv</t>
+  </si>
+  <si>
+    <t>TAGLino is treatd as a "substrate", and Lino.Blood-&gt;TAGLino should not be included in the network</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>13C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
+    </r>
+  </si>
+  <si>
     <r>
       <t>13CLinoKin</t>
     </r>
@@ -1589,20 +1638,175 @@
         <b/>
         <sz val="12"/>
         <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>A</t>
     </r>
   </si>
   <si>
     <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>E</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>F</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>G</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>H</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>I</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13CLinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>J</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>13C</t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>LinoKin</t>
     </r>
@@ -1611,28 +1815,41 @@
         <b/>
         <sz val="12"/>
         <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
     </r>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>13C</t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>LinoKin</t>
     </r>
@@ -1641,28 +1858,41 @@
         <b/>
         <sz val="12"/>
         <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>B</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
     </r>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>13C</t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>LinoKin</t>
     </r>
@@ -1671,28 +1901,41 @@
         <b/>
         <sz val="12"/>
         <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
     </r>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>13C</t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>LinoKin</t>
     </r>
@@ -1701,28 +1944,84 @@
         <b/>
         <sz val="12"/>
         <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>D</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-&gt; AcCoA.Lv</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>13C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>F</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
     </r>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>13C</t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>LinoKin</t>
     </r>
@@ -1731,7 +2030,95 @@
         <b/>
         <sz val="12"/>
         <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>G</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>13C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>H</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>13C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LinoKin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>I</t>
     </r>
@@ -1739,379 +2126,54 @@
       <rPr>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
     </r>
   </si>
   <si>
     <r>
-      <t>13CLinoKin</t>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>13C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LinoKin</t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="12"/>
         <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>B</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>C</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>D</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>H</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>I</t>
-    </r>
-  </si>
-  <si>
-    <t>TAGLino.Lv -&gt; AcCoA.Lv</t>
-  </si>
-  <si>
-    <t>TAGLino is treatd as a "substrate", and Lino.Blood-&gt;TAGLino should not be included in the network</t>
-  </si>
-  <si>
-    <r>
-      <t>13C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>LinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>H</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">J </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
       <t>-&gt; AcCoA.Lv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>LinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>O</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>LinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>P</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>LinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>Q</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>LinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>R</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>LinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>LinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>T</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> -&gt; AcCoA.Lv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>O</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>P</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>Q</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>R</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>S</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>13CLinoKin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>T</t>
     </r>
   </si>
 </sst>
@@ -2119,7 +2181,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2225,14 +2287,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF00B0F0"/>
-      <name val="Aptos Narrow (Body)"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1" tint="0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2600,7 +2664,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2993,16 +3057,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3255A141-2CCB-574F-8A5D-811344C87C12}">
   <dimension ref="A1:J101"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="16.5" thickBot="1">
       <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
@@ -3019,7 +3083,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5">
       <c r="A2" s="23">
         <v>1</v>
       </c>
@@ -3034,7 +3098,7 @@
       </c>
       <c r="E2" s="6"/>
     </row>
-    <row r="3" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="16.5" thickBot="1">
       <c r="A3" s="24">
         <f>A2+1</f>
         <v>2</v>
@@ -3048,7 +3112,7 @@
       <c r="D3" s="30"/>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5">
       <c r="A4" s="24">
         <f t="shared" ref="A4:A68" si="0">A3+1</f>
         <v>3</v>
@@ -3062,7 +3126,7 @@
       <c r="D4" s="30"/>
       <c r="E4" s="6"/>
     </row>
-    <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="16.5" thickBot="1">
       <c r="A5" s="24">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -3076,7 +3140,7 @@
       <c r="D5" s="31"/>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5">
       <c r="A6" s="24">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -3092,7 +3156,7 @@
       </c>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5">
       <c r="A7" s="24">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -3106,7 +3170,7 @@
       <c r="D7" s="62"/>
       <c r="E7" s="6"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5">
       <c r="A8" s="24">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -3120,7 +3184,7 @@
       <c r="D8" s="62"/>
       <c r="E8" s="6"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5">
       <c r="A9" s="24">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -3136,7 +3200,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5">
       <c r="A10" s="24">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -3152,7 +3216,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5">
       <c r="A11" s="24">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -3168,23 +3232,23 @@
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5">
       <c r="A12" s="24">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B12" s="56" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C12" s="57" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="62"/>
       <c r="E12" s="58" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13" s="24">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -3200,7 +3264,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5">
       <c r="A14" s="24">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -3214,7 +3278,7 @@
       <c r="D14" s="62"/>
       <c r="E14" s="6"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5">
       <c r="A15" s="24">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -3228,7 +3292,7 @@
       <c r="D15" s="62"/>
       <c r="E15" s="6"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5">
       <c r="A16" s="24">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -3242,7 +3306,7 @@
       <c r="D16" s="62"/>
       <c r="E16" s="6"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5">
       <c r="A17" s="24">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -3256,7 +3320,7 @@
       <c r="D17" s="62"/>
       <c r="E17" s="6"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5">
       <c r="A18" s="24">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -3270,7 +3334,7 @@
       <c r="D18" s="62"/>
       <c r="E18" s="6"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5">
       <c r="A19" s="24">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -3284,7 +3348,7 @@
       <c r="D19" s="62"/>
       <c r="E19" s="6"/>
     </row>
-    <row r="20" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="16.5" thickBot="1">
       <c r="A20" s="24">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -3300,7 +3364,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5">
       <c r="A21" s="24">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -3318,7 +3382,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5">
       <c r="A22" s="24">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3334,7 +3398,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5">
       <c r="A23" s="24">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3348,7 +3412,7 @@
       <c r="D23" s="65"/>
       <c r="E23" s="6"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5">
       <c r="A24" s="24">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3362,7 +3426,7 @@
       <c r="D24" s="65"/>
       <c r="E24" s="6"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5">
       <c r="A25" s="24">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3376,7 +3440,7 @@
       <c r="D25" s="65"/>
       <c r="E25" s="6"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5">
       <c r="A26" s="24">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3390,7 +3454,7 @@
       <c r="D26" s="65"/>
       <c r="E26" s="6"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5">
       <c r="A27" s="24">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3404,7 +3468,7 @@
       <c r="D27" s="65"/>
       <c r="E27" s="6"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5">
       <c r="A28" s="24">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3418,7 +3482,7 @@
       <c r="D28" s="65"/>
       <c r="E28" s="6"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5">
       <c r="A29" s="24">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3432,7 +3496,7 @@
       <c r="D29" s="65"/>
       <c r="E29" s="6"/>
     </row>
-    <row r="30" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="16.5" thickBot="1">
       <c r="A30" s="24">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3446,7 +3510,7 @@
       <c r="D30" s="66"/>
       <c r="E30" s="6"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5">
       <c r="A31" s="24">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -3462,7 +3526,7 @@
       </c>
       <c r="E31" s="6"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5">
       <c r="A32" s="24">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -3476,7 +3540,7 @@
       <c r="D32" s="37"/>
       <c r="E32" s="6"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5">
       <c r="A33" s="24">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -3490,7 +3554,7 @@
       <c r="D33" s="37"/>
       <c r="E33" s="6"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5">
       <c r="A34" s="24">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -3504,7 +3568,7 @@
       <c r="D34" s="37"/>
       <c r="E34" s="6"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5">
       <c r="A35" s="24">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -3518,7 +3582,7 @@
       <c r="D35" s="37"/>
       <c r="E35" s="6"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5">
       <c r="A36" s="24">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -3532,7 +3596,7 @@
       <c r="D36" s="37"/>
       <c r="E36" s="6"/>
     </row>
-    <row r="37" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" ht="16.5" thickBot="1">
       <c r="A37" s="24">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -3546,7 +3610,7 @@
       <c r="D37" s="40"/>
       <c r="E37" s="6"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5">
       <c r="A38" s="24">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -3562,7 +3626,7 @@
       </c>
       <c r="E38" s="6"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5">
       <c r="A39" s="24">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -3576,7 +3640,7 @@
       <c r="D39" s="68"/>
       <c r="E39" s="6"/>
     </row>
-    <row r="40" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5">
       <c r="A40" s="24">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -3590,7 +3654,7 @@
       <c r="D40" s="68"/>
       <c r="E40" s="6"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5">
       <c r="A41" s="24">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -3604,7 +3668,7 @@
       <c r="D41" s="68"/>
       <c r="E41" s="6"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5">
       <c r="A42" s="24">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -3618,7 +3682,7 @@
       <c r="D42" s="68"/>
       <c r="E42" s="6"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5">
       <c r="A43" s="24">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -3632,7 +3696,7 @@
       <c r="D43" s="68"/>
       <c r="E43" s="6"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5">
       <c r="A44" s="24">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -3646,7 +3710,7 @@
       <c r="D44" s="68"/>
       <c r="E44" s="6"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5">
       <c r="A45" s="24">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -3660,7 +3724,7 @@
       <c r="D45" s="68"/>
       <c r="E45" s="6"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5">
       <c r="A46" s="24">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -3674,7 +3738,7 @@
       <c r="D46" s="68"/>
       <c r="E46" s="6"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5">
       <c r="A47" s="24">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -3688,7 +3752,7 @@
       <c r="D47" s="68"/>
       <c r="E47" s="6"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5">
       <c r="A48" s="24">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -3702,7 +3766,7 @@
       <c r="D48" s="68"/>
       <c r="E48" s="6"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5">
       <c r="A49" s="24">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -3716,7 +3780,7 @@
       <c r="D49" s="68"/>
       <c r="E49" s="6"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5">
       <c r="A50" s="24">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -3730,7 +3794,7 @@
       <c r="D50" s="68"/>
       <c r="E50" s="6"/>
     </row>
-    <row r="51" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" ht="16.5" thickBot="1">
       <c r="A51" s="24">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -3744,7 +3808,7 @@
       <c r="D51" s="69"/>
       <c r="E51" s="6"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5">
       <c r="A52" s="24">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -3760,7 +3824,7 @@
       </c>
       <c r="E52" s="6"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5">
       <c r="A53" s="24">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -3774,7 +3838,7 @@
       <c r="D53" s="62"/>
       <c r="E53" s="6"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5">
       <c r="A54" s="24">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -3788,7 +3852,7 @@
       <c r="D54" s="62"/>
       <c r="E54" s="6"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5">
       <c r="A55" s="24">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -3802,7 +3866,7 @@
       <c r="D55" s="62"/>
       <c r="E55" s="6"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5">
       <c r="A56" s="24">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -3816,7 +3880,7 @@
       <c r="D56" s="62"/>
       <c r="E56" s="6"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5">
       <c r="A57" s="24">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -3830,7 +3894,7 @@
       <c r="D57" s="62"/>
       <c r="E57" s="6"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5">
       <c r="A58" s="24">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -3844,7 +3908,7 @@
       <c r="D58" s="62"/>
       <c r="E58" s="6"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5">
       <c r="A59" s="24">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -3858,7 +3922,7 @@
       <c r="D59" s="62"/>
       <c r="E59" s="6"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5">
       <c r="A60" s="24">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -3872,7 +3936,7 @@
       <c r="D60" s="62"/>
       <c r="E60" s="6"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5">
       <c r="A61" s="24">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -3886,7 +3950,7 @@
       <c r="D61" s="62"/>
       <c r="E61" s="6"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5">
       <c r="A62" s="24">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -3900,7 +3964,7 @@
       <c r="D62" s="62"/>
       <c r="E62" s="6"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5">
       <c r="A63" s="24">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -3914,7 +3978,7 @@
       <c r="D63" s="62"/>
       <c r="E63" s="6"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5">
       <c r="A64" s="24">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -3928,7 +3992,7 @@
       <c r="D64" s="62"/>
       <c r="E64" s="6"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5">
       <c r="A65" s="24">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -3942,7 +4006,7 @@
       <c r="D65" s="62"/>
       <c r="E65" s="6"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5">
       <c r="A66" s="24">
         <f t="shared" si="0"/>
         <v>65</v>
@@ -3956,7 +4020,7 @@
       <c r="D66" s="62"/>
       <c r="E66" s="6"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5">
       <c r="A67" s="24">
         <f t="shared" si="0"/>
         <v>66</v>
@@ -3970,7 +4034,7 @@
       <c r="D67" s="62"/>
       <c r="E67" s="6"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:5">
       <c r="A68" s="24">
         <f t="shared" si="0"/>
         <v>67</v>
@@ -3984,7 +4048,7 @@
       <c r="D68" s="62"/>
       <c r="E68" s="6"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5">
       <c r="A69" s="24">
         <f t="shared" ref="A69:A101" si="1">A68+1</f>
         <v>68</v>
@@ -3998,7 +4062,7 @@
       <c r="D69" s="62"/>
       <c r="E69" s="6"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5">
       <c r="A70" s="24">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -4012,7 +4076,7 @@
       <c r="D70" s="62"/>
       <c r="E70" s="6"/>
     </row>
-    <row r="71" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" ht="16.5" thickBot="1">
       <c r="A71" s="24">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -4026,7 +4090,7 @@
       <c r="D71" s="63"/>
       <c r="E71" s="6"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5">
       <c r="A72" s="24">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -4042,7 +4106,7 @@
       </c>
       <c r="E72" s="6"/>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5">
       <c r="A73" s="24">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -4056,7 +4120,7 @@
       <c r="D73" s="62"/>
       <c r="E73" s="8"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5">
       <c r="A74" s="24">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -4070,7 +4134,7 @@
       <c r="D74" s="62"/>
       <c r="E74" s="6"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5">
       <c r="A75" s="24">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -4084,7 +4148,7 @@
       <c r="D75" s="62"/>
       <c r="E75" s="6"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5">
       <c r="A76" s="24">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -4098,7 +4162,7 @@
       <c r="D76" s="62"/>
       <c r="E76" s="6"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5">
       <c r="A77" s="24">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -4112,7 +4176,7 @@
       <c r="D77" s="62"/>
       <c r="E77" s="6"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5">
       <c r="A78" s="24">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -4128,7 +4192,7 @@
       </c>
       <c r="E78" s="6"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5">
       <c r="A79" s="24">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -4142,7 +4206,7 @@
       <c r="D79" s="62"/>
       <c r="E79" s="6"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5">
       <c r="A80" s="24">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -4156,7 +4220,7 @@
       <c r="D80" s="62"/>
       <c r="E80" s="6"/>
     </row>
-    <row r="81" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" ht="16.5" thickBot="1">
       <c r="A81" s="24">
         <f t="shared" si="1"/>
         <v>80</v>
@@ -4170,7 +4234,7 @@
       <c r="D81" s="62"/>
       <c r="E81" s="6"/>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5">
       <c r="A82" s="24">
         <f t="shared" si="1"/>
         <v>81</v>
@@ -4188,7 +4252,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" ht="16.5" thickBot="1">
       <c r="A83" s="24">
         <f t="shared" si="1"/>
         <v>82</v>
@@ -4202,7 +4266,7 @@
       <c r="D83" s="39"/>
       <c r="E83" s="6"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5">
       <c r="A84" s="24">
         <f t="shared" si="1"/>
         <v>83</v>
@@ -4218,7 +4282,7 @@
       </c>
       <c r="E84" s="6"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5">
       <c r="A85" s="24">
         <f t="shared" si="1"/>
         <v>84</v>
@@ -4232,7 +4296,7 @@
       <c r="D85" s="62"/>
       <c r="E85" s="6"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5">
       <c r="A86" s="24">
         <f t="shared" si="1"/>
         <v>85</v>
@@ -4246,7 +4310,7 @@
       <c r="D86" s="62"/>
       <c r="E86" s="6"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5">
       <c r="A87" s="24">
         <f t="shared" si="1"/>
         <v>86</v>
@@ -4260,7 +4324,7 @@
       <c r="D87" s="62"/>
       <c r="E87" s="6"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5">
       <c r="A88" s="24">
         <f t="shared" si="1"/>
         <v>87</v>
@@ -4274,7 +4338,7 @@
       <c r="D88" s="62"/>
       <c r="E88" s="6"/>
     </row>
-    <row r="89" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" ht="16.5" thickBot="1">
       <c r="A89" s="24">
         <f t="shared" si="1"/>
         <v>88</v>
@@ -4288,7 +4352,7 @@
       <c r="D89" s="63"/>
       <c r="E89" s="6"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5">
       <c r="A90" s="24">
         <f t="shared" si="1"/>
         <v>89</v>
@@ -4304,7 +4368,7 @@
       </c>
       <c r="E90" s="6"/>
     </row>
-    <row r="91" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" ht="16.5" thickBot="1">
       <c r="A91" s="24">
         <f t="shared" si="1"/>
         <v>90</v>
@@ -4318,7 +4382,7 @@
       <c r="D91" s="63"/>
       <c r="E91" s="6"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5">
       <c r="A92" s="24">
         <f t="shared" si="1"/>
         <v>91</v>
@@ -4333,7 +4397,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:5">
       <c r="A93" s="24">
         <f t="shared" si="1"/>
         <v>92</v>
@@ -4346,7 +4410,7 @@
       </c>
       <c r="D93" s="62"/>
     </row>
-    <row r="94" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" ht="16.5" thickBot="1">
       <c r="A94" s="24">
         <f t="shared" si="1"/>
         <v>93</v>
@@ -4359,7 +4423,7 @@
       </c>
       <c r="D94" s="63"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:5">
       <c r="A95" s="24">
         <f t="shared" si="1"/>
         <v>94</v>
@@ -4374,7 +4438,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:5">
       <c r="A96" s="24">
         <f t="shared" si="1"/>
         <v>95</v>
@@ -4387,7 +4451,7 @@
       </c>
       <c r="D96" s="62"/>
     </row>
-    <row r="97" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" ht="16.5" thickBot="1">
       <c r="A97" s="24">
         <f t="shared" si="1"/>
         <v>96</v>
@@ -4400,7 +4464,7 @@
       </c>
       <c r="D97" s="63"/>
     </row>
-    <row r="98" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" ht="16.5" thickBot="1">
       <c r="A98" s="24">
         <f t="shared" si="1"/>
         <v>97</v>
@@ -4416,7 +4480,7 @@
       </c>
       <c r="E98" s="6"/>
     </row>
-    <row r="99" spans="1:10" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" ht="17.100000000000001" customHeight="1" thickBot="1">
       <c r="A99" s="24">
         <f t="shared" si="1"/>
         <v>98</v>
@@ -4437,7 +4501,7 @@
       <c r="I99" s="60"/>
       <c r="J99" s="60"/>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:10">
       <c r="A100" s="24">
         <f t="shared" si="1"/>
         <v>99</v>
@@ -4452,7 +4516,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10">
       <c r="A101" s="24">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -4488,16 +4552,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6AE8287-079C-D041-8E27-642CD2612D07}">
-  <dimension ref="A1:D32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="3.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultColWidth="3.375" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4511,7 +4575,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" s="1">
         <f>COUNT(LvM!A1:A188) + 1</f>
         <v>101</v>
@@ -4526,7 +4590,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3" s="3">
         <f>A2</f>
         <v>101</v>
@@ -4541,9 +4605,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" s="3">
-        <f t="shared" ref="A4:A32" si="0">A3</f>
+        <f t="shared" ref="A4:A30" si="0">A3</f>
         <v>101</v>
       </c>
       <c r="B4" s="11" t="s">
@@ -4556,7 +4620,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4571,7 +4635,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4586,7 +4650,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4">
       <c r="A7" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4601,7 +4665,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="16.5" thickBot="1">
       <c r="A8" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4616,7 +4680,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4">
       <c r="A9" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4631,7 +4695,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4">
       <c r="A10" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4646,7 +4710,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4">
       <c r="A11" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4661,7 +4725,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4">
       <c r="A12" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4676,7 +4740,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4">
       <c r="A13" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4691,7 +4755,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4">
       <c r="A14" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4706,7 +4770,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4">
       <c r="A15" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4721,7 +4785,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="16.5" thickBot="1">
       <c r="A16" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4736,7 +4800,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4">
       <c r="A17" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4751,7 +4815,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4">
       <c r="A18" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4766,7 +4830,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4">
       <c r="A19" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4781,7 +4845,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4">
       <c r="A20" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -4796,184 +4860,154 @@
         <v>174</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4">
       <c r="A21" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="B21" t="s">
+        <v>189</v>
+      </c>
+      <c r="C21" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="B22" t="s">
+        <v>200</v>
+      </c>
+      <c r="C22" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="3">
+        <f t="shared" si="0"/>
+        <v>101</v>
+      </c>
+      <c r="B23" t="s">
+        <v>201</v>
+      </c>
+      <c r="C23" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="3">
+        <f t="shared" si="0"/>
+        <v>101</v>
+      </c>
+      <c r="B24" t="s">
+        <v>202</v>
+      </c>
+      <c r="C24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="3">
+    <row r="25" spans="1:4">
+      <c r="A25" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="B25" t="s">
+        <v>203</v>
+      </c>
+      <c r="C25" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D25" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
+    <row r="26" spans="1:4">
+      <c r="A26" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="C24" s="1" t="s">
+      <c r="B26" t="s">
+        <v>204</v>
+      </c>
+      <c r="C26" t="s">
         <v>16</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D26" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
+    <row r="27" spans="1:4">
+      <c r="A27" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="B27" t="s">
+        <v>205</v>
+      </c>
+      <c r="C27" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D27" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="3">
+    <row r="28" spans="1:4">
+      <c r="A28" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B26" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="B28" t="s">
+        <v>206</v>
+      </c>
+      <c r="C28" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D28" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="3">
+    <row r="29" spans="1:4">
+      <c r="A29" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="C27" s="1" t="s">
+      <c r="B29" t="s">
+        <v>207</v>
+      </c>
+      <c r="C29" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="3">
+      <c r="D29" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="3">
         <f t="shared" si="0"/>
         <v>101</v>
       </c>
-      <c r="B28" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="C28" s="1" t="s">
+      <c r="B30" t="s">
+        <v>208</v>
+      </c>
+      <c r="C30" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="3">
-        <f t="shared" si="0"/>
-        <v>101</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="3">
-        <f t="shared" si="0"/>
-        <v>101</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="3">
-        <f t="shared" si="0"/>
-        <v>101</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="3">
-        <f t="shared" si="0"/>
-        <v>101</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>212</v>
+      <c r="D30" t="s">
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>